<commit_message>
docs(prds): exclui cards Matriz FG e Manifestacao do Destinatario; corrige vinculo de Inconsistencias
Saem do hub, da secao Documentacao e Contextualizacao, os cards
"Matriz FG — Validacoes e Configuracoes" e "Manifestacao do
Destinatario". Os documentos de origem (artefatos externos) nao foram
tocados.

Correcao na priorizacao: as nove funcionalidades de Inconsistencias
apontavam para o artefato da Matriz FG, tomado por engano como PRD do
modulo durante a curadoria. O modulo nao tem PRD publicado - o card
segue em rascunho - e elas passam a declarar sem PRD no Mapa
detalhado. Vinculos: 142 com bloco ou secao, 8 lacunas em PRD
existente, 34 sem PRD.

Changelog R-068.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/docs/priorizacao-mvp.xlsx
+++ b/docs/docs/priorizacao-mvp.xlsx
@@ -2757,9 +2757,9 @@
           <t>Toda inconsistência tem vínculo obrigatório ao DF de origem. O campo rfId é opcional: nulo para inconsistências geradas antes da criação dos RFs (falhas de ingestão); preenchido quando a inconsistência é específica de um RF já criado (pós-apuração ou pós-conciliação financeira).</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>PRD do módulo, publicado à parte</t>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>Sem PRD</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -2808,9 +2808,9 @@
           <t>Um mesmo DF pode acumular inconsistências geradas em etapas distintas do ciclo de vida (ex: divergência de valor IBS na apuração E comprovante CBS ausente na conciliação). Todas exibidas simultaneamente como pills nas listagens.</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>PRD do módulo, publicado à parte</t>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>Sem PRD</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -2859,9 +2859,9 @@
           <t>Inconsistências de apuração identificadas individualmente por imposto: capur_ibs_valor (valor divergente), capur_ibs_aliquota (alíquota divergente), capur_cbs_valor, capur_cbs_aliquota. IBS e CBS apurados de forma independente.</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>PRD do módulo, publicado à parte</t>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>Sem PRD</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -2910,9 +2910,9 @@
           <t>Inconsistências financeiras identificadas por imposto: cfin_ibs_split (split não executado), cfin_ibs_comprovante (comprovante divergente), cfin_cbs_split, cfin_cbs_comprovante. Inclui "Sem Comprovante" para contratos RAD sem anexo.</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>PRD do módulo, publicado à parte</t>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>Sem PRD</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -2961,9 +2961,9 @@
           <t>Quadro kanban com colunas: Aberta, Em Análise, Aguardando Emitente, Resolvida e Glosada. Cards movidos entre colunas registram data e usuário da transição.</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>PRD do módulo, publicado à parte</t>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>Sem PRD</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -3012,9 +3012,9 @@
           <t>Card de inconsistência pode ser atribuído a um operador específico, com campo de responsável e registro de data de atribuição.</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>PRD do módulo, publicado à parte</t>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>Sem PRD</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -3071,9 +3071,9 @@
           <t>Modal expandido em dois painéis: dados da inconsistência e ações sugeridas à esquerda; histórico cronológico completo de transições, atribuições e comentários à direita.</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>PRD do módulo, publicado à parte</t>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>Sem PRD</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -3122,9 +3122,9 @@
           <t>Assistente de diagnóstico com perguntas sequenciais para identificar o tipo de inconsistência: fluxo de entrada ou saída? Etapa de apuração (CAPUR) ou financeira (CFIN)? Qual imposto (IBS ou CBS)?</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
-        <is>
-          <t>PRD do módulo, publicado à parte</t>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>Sem PRD</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -3173,9 +3173,9 @@
           <t>Filtros combinados por tipo de inconsistência (taxonomia CAPUR/CFIN) e DF de origem, com suporte a seleção múltipla.</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>PRD do módulo, publicado à parte</t>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>Sem PRD</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -10743,125 +10743,116 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F90" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F92" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F93" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F97" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F100" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F103" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F106" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F122" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F123" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F124" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F125" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F126" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F127" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F128" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F129" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F130" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F131" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F132" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F133" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F134" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F135" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F136" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F137" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F138" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F139" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F140" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F141" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F142" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F143" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F144" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F145" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F146" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F147" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F148" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F149" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F150" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F151" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F152" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F157" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F158" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F159" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F160" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F161" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F162" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F163" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F172" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F173" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F178" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F180" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F182" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F183" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F185" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F90" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F92" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F93" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F97" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F100" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F103" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F106" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F122" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F123" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F124" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F125" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F126" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F127" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F128" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F129" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F130" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F131" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F132" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F133" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F134" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F135" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F136" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F137" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F138" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F139" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F140" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F141" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F142" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F143" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F144" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F145" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F146" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F147" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F148" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F149" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F150" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F151" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F152" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F157" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F158" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F159" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F160" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F161" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F162" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F163" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F172" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F173" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F178" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F180" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F182" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F183" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F185" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId150"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(prds): changelog — mapa v2.9, priorizacao v2.10, proposta de usuarios v1.2 (R-246..R-248)
Mapa: Usuarios e Acessos segue a gestao implementada (historico do
usuario, redefinicao de senha, filtro por situacao); as quatro da
parcialidade saem de NOVAS e entram em Creditos. Priorizacao: M0 segue
117, D20 em aberto (login proprio no M0, SSO em M1). Proposta: detalhe
da D-USR-05, D-USR-06 e tempos de sessao.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/docs/priorizacao-mvp.xlsx
+++ b/docs/docs/priorizacao-mvp.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Como revisar" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Priorização'!$A$1:$O$294</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Priorização'!$A$1:$O$296</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Revisões'!$A$1:$H$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O294"/>
+  <dimension ref="A1:O296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2139,9 +2139,9 @@
           <t>Risco/Inc.</t>
         </is>
       </c>
-      <c r="H30" s="11" t="inlineStr">
-        <is>
-          <t>Nova</t>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -2190,9 +2190,9 @@
           <t>Listagem</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
-        <is>
-          <t>Nova</t>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Um painel por tributo, com a partição, a conferência da soma, o prazo do art. 54 mais próximo e a última leitura do órgão.</t>
+          <t>Quadro CBS × IBS com os registros fiscais e as parcelas de cada tributo, a conferência da soma, o prazo do art. 54 mais próximo e a última leitura do órgão. O mesmo quadro serve ao detalhe do RF.</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -2241,9 +2241,9 @@
           <t>Listagem</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr">
-        <is>
-          <t>Nova</t>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Razão do RF: cada movimento leva uma quantia de uma parcela para outra, com causa, fonte e vínculo. É a fonte da partição — a soma dos movimentos é o saldo de cada parcela.</t>
+          <t>Razão do RF: cada movimento leva uma quantia de uma parcela para outra, com causa, fonte e vínculo, numa trilha de auditoria filtrável. A soma dos movimentos é o saldo de cada parcela.</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -2292,9 +2292,9 @@
           <t>Listagem</t>
         </is>
       </c>
-      <c r="H33" s="11" t="inlineStr">
-        <is>
-          <t>Nova</t>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -14534,12 +14534,12 @@
       </c>
       <c r="E270" s="4" t="inlineStr">
         <is>
-          <t>Usuário, e-mail, perfil, último acesso e situação, com o total de ativos, administradores, convites pendentes e inativos.</t>
-        </is>
-      </c>
-      <c r="F270" s="12" t="inlineStr">
-        <is>
-          <t>Sem PRD</t>
+          <t>Usuário, e-mail, perfil, último acesso e situação, com busca e filtro por perfil. Os indicadores contam ativos, administradores, convites pendentes e quem está sem acesso há 90 dias, candidato à revisão de acessos.</t>
+        </is>
+      </c>
+      <c r="F270" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G270" s="3" t="inlineStr">
@@ -14585,12 +14585,12 @@
       </c>
       <c r="E271" s="4" t="inlineStr">
         <is>
-          <t>Administrador, Analista Fiscal, Controller e Auditor, cada um com o alcance declarado por módulo e a permissão de agir ou só ler.</t>
-        </is>
-      </c>
-      <c r="F271" s="12" t="inlineStr">
-        <is>
-          <t>Sem PRD</t>
+          <t>Um perfil por usuário, válido em toda a organização. Só o administrador troca o perfil, sempre com motivo, e ninguém altera o próprio.</t>
+        </is>
+      </c>
+      <c r="F271" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G271" s="3" t="inlineStr">
@@ -14636,12 +14636,12 @@
       </c>
       <c r="E272" s="4" t="inlineStr">
         <is>
-          <t>Convida por e-mail com o perfil já definido, e reenvia o convite que não foi aceito.</t>
-        </is>
-      </c>
-      <c r="F272" s="12" t="inlineStr">
-        <is>
-          <t>Sem PRD</t>
+          <t>Convida por e-mail com o perfil já definido. O convite vale 7 dias e, pelo link, a pessoa cria a própria senha no primeiro acesso; o vencido pode ser reenviado, com link novo, ou cancelado.</t>
+        </is>
+      </c>
+      <c r="F272" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G272" s="3" t="inlineStr">
@@ -14687,12 +14687,12 @@
       </c>
       <c r="E273" s="4" t="inlineStr">
         <is>
-          <t>Corta o acesso sem apagar o usuário, preservando a trilha do que ele fez, e devolve o acesso quando necessário.</t>
-        </is>
-      </c>
-      <c r="F273" s="12" t="inlineStr">
-        <is>
-          <t>Sem PRD</t>
+          <t>Desativa sem apagar o usuário, com motivo, preservando a trilha do que ele fez, e reativa com o perfil anterior. O último administrador ativo não pode ser desativado.</t>
+        </is>
+      </c>
+      <c r="F273" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G273" s="3" t="inlineStr">
@@ -14733,17 +14733,17 @@
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>Abas por situação do acesso</t>
+          <t>Filtro por situação do acesso</t>
         </is>
       </c>
       <c r="E274" s="4" t="inlineStr">
         <is>
-          <t>Todos, ativos, pendentes e inativos, para achar rápido quem está sem acesso ou com convite parado.</t>
-        </is>
-      </c>
-      <c r="F274" s="12" t="inlineStr">
-        <is>
-          <t>Sem PRD</t>
+          <t>Ativo, convite pendente, convite vencido e inativo, para achar rápido quem está sem acesso ou com convite parado.</t>
+        </is>
+      </c>
+      <c r="F274" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G274" s="3" t="inlineStr">
@@ -14844,12 +14844,12 @@
       </c>
       <c r="E276" s="4" t="inlineStr">
         <is>
-          <t>Administrador, Fiscal, Tesouraria, Leitura e Fornecedor. O perfil de Tesouraria é pressuposto pelo Ressarcimento e não existia no cadastro.</t>
+          <t>Administrador, Fiscal, Tesouraria, Leitura e Fornecedor, cada um com o que pode fazer, na tela de usuários e no próprio convite. O perfil de Tesouraria é pressuposto pelo Ressarcimento e não existia no cadastro.</t>
         </is>
       </c>
       <c r="F276" s="5" t="inlineStr">
         <is>
-          <t>PRD de Organização</t>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G276" s="3" t="inlineStr">
@@ -14895,12 +14895,12 @@
       </c>
       <c r="E277" s="4" t="inlineStr">
         <is>
-          <t>Revogar sem encerrar a sessão deixa uma janela em que o acesso revogado continua valendo.</t>
+          <t>Desativar encerra as sessões abertas na hora, e o administrador também pode encerrá-las sem desativar. Sem isso, o acesso revogado continua valendo até a sessão expirar.</t>
         </is>
       </c>
       <c r="F277" s="5" t="inlineStr">
         <is>
-          <t>PRD de Organização</t>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G277" s="3" t="inlineStr">
@@ -15033,27 +15033,27 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>Operacional</t>
+          <t>Gestão</t>
         </is>
       </c>
       <c r="C280" s="3" t="inlineStr">
         <is>
-          <t>Ressarcimento</t>
+          <t>Usuários e Acessos</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>Saldo credor por período e tributo</t>
+          <t>Histórico do usuário</t>
         </is>
       </c>
       <c r="E280" s="4" t="inlineStr">
         <is>
-          <t>Por período e por tributo, na matriz: saldo inicial, apropriado, compensado, saldo credor, o que saiu para ressarcimento e o transportado. É a base da decisão de compensar ou pedir o dinheiro.</t>
+          <t>Convite, aceite, troca de perfil, desativação, reativação e sessões encerradas, com autor, data e motivo. Responde quem deu ou tirou um acesso, e por quê.</t>
         </is>
       </c>
       <c r="F280" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-01 Ver o saldo credor do tributo</t>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G280" s="3" t="inlineStr">
@@ -15084,32 +15084,32 @@
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>Operacional</t>
+          <t>Gestão</t>
         </is>
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>Ressarcimento</t>
+          <t>Usuários e Acessos</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>Comparar compensar e ressarcir</t>
+          <t>Redefinição de senha pelo administrador</t>
         </is>
       </c>
       <c r="E281" s="4" t="inlineStr">
         <is>
-          <t>Para o período em curso, as duas hipóteses lado a lado: uso do saldo, quando o dinheiro volta e a correção estimada pela Selic.</t>
+          <t>Envia ao usuário um link de uso único para criar senha nova. O administrador nunca vê nem define a senha de outra pessoa.</t>
         </is>
       </c>
       <c r="F281" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-02 Comparar compensar e ressarcir</t>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G281" s="3" t="inlineStr">
         <is>
-          <t>Analítico</t>
+          <t>Ação</t>
         </is>
       </c>
       <c r="H281" s="3" t="inlineStr">
@@ -15117,9 +15117,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I281" s="9" t="inlineStr">
-        <is>
-          <t>M2</t>
+      <c r="I281" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
         </is>
       </c>
       <c r="J281" s="3" t="inlineStr"/>
@@ -15145,22 +15145,22 @@
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>Declarar e cancelar a intenção</t>
+          <t>Saldo credor por período e tributo</t>
         </is>
       </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
-          <t>Intenção do tributo até o último dia útil do período, com o efeito mostrado antes e aprovação acima do limite. Reserva o saldo; cancelada ou vencida, o saldo volta a compensar.</t>
+          <t>Por período e por tributo, na matriz: saldo inicial, apropriado, compensado, saldo credor, o que saiu para ressarcimento e o transportado. É a base da decisão de compensar ou pedir o dinheiro.</t>
         </is>
       </c>
       <c r="F282" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-03 Declarar e cancelar a intenção</t>
+          <t>PRD de Ressarcimento · F-01 Ver o saldo credor do tributo</t>
         </is>
       </c>
       <c r="G282" s="3" t="inlineStr">
         <is>
-          <t>Ação</t>
+          <t>Listagem</t>
         </is>
       </c>
       <c r="H282" s="3" t="inlineStr">
@@ -15196,22 +15196,22 @@
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>Montar o pedido de CBS por documento</t>
+          <t>Comparar compensar e ressarcir</t>
         </is>
       </c>
       <c r="E283" s="4" t="inlineStr">
         <is>
-          <t>Escolhe os documentos do saldo reservado que entram no pedido. O que fica de fora volta a compensar desde a data do pedido.</t>
+          <t>Para o período em curso, as duas hipóteses lado a lado: uso do saldo, quando o dinheiro volta e a correção estimada pela Selic.</t>
         </is>
       </c>
       <c r="F283" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-04 Montar o pedido de CBS</t>
+          <t>PRD de Ressarcimento · F-02 Comparar compensar e ressarcir</t>
         </is>
       </c>
       <c r="G283" s="3" t="inlineStr">
         <is>
-          <t>Ação</t>
+          <t>Analítico</t>
         </is>
       </c>
       <c r="H283" s="3" t="inlineStr">
@@ -15219,9 +15219,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I283" s="10" t="inlineStr">
-        <is>
-          <t>M1</t>
+      <c r="I283" s="9" t="inlineStr">
+        <is>
+          <t>M2</t>
         </is>
       </c>
       <c r="J283" s="3" t="inlineStr"/>
@@ -15247,17 +15247,17 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>Registrar o pedido de CBS (PER/DCOMP)</t>
+          <t>Declarar e cancelar a intenção</t>
         </is>
       </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
-          <t>Número do PER/DCOMP e data de transmissão. Calcula o fim da análise e a data do pagamento por silêncio do Fisco.</t>
+          <t>Intenção do tributo até o último dia útil do período, com o efeito mostrado antes e aprovação acima do limite. Reserva o saldo; cancelada ou vencida, o saldo volta a compensar.</t>
         </is>
       </c>
       <c r="F284" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-05 Registrar o pedido de CBS</t>
+          <t>PRD de Ressarcimento · F-03 Declarar e cancelar a intenção</t>
         </is>
       </c>
       <c r="G284" s="3" t="inlineStr">
@@ -15298,22 +15298,22 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>Listagem de pedidos do tributo</t>
+          <t>Montar o pedido de CBS por documento</t>
         </is>
       </c>
       <c r="E285" s="4" t="inlineStr">
         <is>
-          <t>Pedidos com identificador no órgão, valor, prazo, contagem regressiva, situação e valor deferido.</t>
+          <t>Escolhe os documentos do saldo reservado que entram no pedido. O que fica de fora volta a compensar desde a data do pedido.</t>
         </is>
       </c>
       <c r="F285" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-06 Listar os pedidos do tributo</t>
+          <t>PRD de Ressarcimento · F-04 Montar o pedido de CBS</t>
         </is>
       </c>
       <c r="G285" s="3" t="inlineStr">
         <is>
-          <t>Listagem</t>
+          <t>Ação</t>
         </is>
       </c>
       <c r="H285" s="3" t="inlineStr">
@@ -15349,22 +15349,22 @@
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>Acompanhar análise e fiscalização</t>
+          <t>Registrar o pedido de CBS (PER/DCOMP)</t>
         </is>
       </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
-          <t>Fiscalização suspende o prazo e tem limite de 360 dias. Mostra quando o prazo do Fisco se esgota sem manifestação.</t>
+          <t>Número do PER/DCOMP e data de transmissão. Calcula o fim da análise e a data do pagamento por silêncio do Fisco.</t>
         </is>
       </c>
       <c r="F286" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-07 Acompanhar análise, exigência e fiscalização</t>
+          <t>PRD de Ressarcimento · F-05 Registrar o pedido de CBS</t>
         </is>
       </c>
       <c r="G286" s="3" t="inlineStr">
         <is>
-          <t>Risco/Inc.</t>
+          <t>Ação</t>
         </is>
       </c>
       <c r="H286" s="3" t="inlineStr">
@@ -15400,22 +15400,22 @@
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>Registrar decisão e cancelamento</t>
+          <t>Listagem de pedidos do tributo</t>
         </is>
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>Deferido, deferido parcial, indeferido ou cancelado, cada um devolvendo o remanescente à compensação a partir da data que a norma define.</t>
+          <t>Pedidos com identificador no órgão, valor, prazo, contagem regressiva, situação e valor deferido.</t>
         </is>
       </c>
       <c r="F287" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-08 Registrar a decisão e o cancelamento</t>
+          <t>PRD de Ressarcimento · F-06 Listar os pedidos do tributo</t>
         </is>
       </c>
       <c r="G287" s="3" t="inlineStr">
         <is>
-          <t>Ação</t>
+          <t>Listagem</t>
         </is>
       </c>
       <c r="H287" s="3" t="inlineStr">
@@ -15451,22 +15451,22 @@
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>Conciliar o recebimento com Selic</t>
+          <t>Acompanhar análise e fiscalização</t>
         </is>
       </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
-          <t>Recebido contra deferido corrigido. Extingue os créditos do pedido com o método Ressarcimento, e só aqui o status do crédito muda.</t>
+          <t>Fiscalização suspende o prazo e tem limite de 360 dias. Mostra quando o prazo do Fisco se esgota sem manifestação.</t>
         </is>
       </c>
       <c r="F288" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-09 Conciliar o recebimento</t>
+          <t>PRD de Ressarcimento · F-07 Acompanhar análise, exigência e fiscalização</t>
         </is>
       </c>
       <c r="G288" s="3" t="inlineStr">
         <is>
-          <t>Ação</t>
+          <t>Risco/Inc.</t>
         </is>
       </c>
       <c r="H288" s="3" t="inlineStr">
@@ -15502,22 +15502,22 @@
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>Previsão de entrada de caixa por tributo</t>
+          <t>Registrar decisão e cancelamento</t>
         </is>
       </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
-          <t>Deferidos e em análise, datados pelo prazo legal, com correção estimada. Uma previsão para CBS e outra para IBS.</t>
+          <t>Deferido, deferido parcial, indeferido ou cancelado, cada um devolvendo o remanescente à compensação a partir da data que a norma define.</t>
         </is>
       </c>
       <c r="F289" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-10 Prever a entrada de caixa do tributo</t>
+          <t>PRD de Ressarcimento · F-08 Registrar a decisão e o cancelamento</t>
         </is>
       </c>
       <c r="G289" s="3" t="inlineStr">
         <is>
-          <t>Analítico</t>
+          <t>Ação</t>
         </is>
       </c>
       <c r="H289" s="3" t="inlineStr">
@@ -15525,9 +15525,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I289" s="9" t="inlineStr">
-        <is>
-          <t>M2</t>
+      <c r="I289" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
         </is>
       </c>
       <c r="J289" s="3" t="inlineStr"/>
@@ -15553,22 +15553,22 @@
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>Alertas de prazo do ressarcimento</t>
+          <t>Conciliar o recebimento com Selic</t>
         </is>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>Intenção, pedido, fim da análise e pagamento por silêncio, por tributo, na tela e como eventos da régua de Automações.</t>
+          <t>Recebido contra deferido corrigido. Extingue os créditos do pedido com o método Ressarcimento, e só aqui o status do crédito muda.</t>
         </is>
       </c>
       <c r="F290" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-11 Alertar os prazos do tributo</t>
+          <t>PRD de Ressarcimento · F-09 Conciliar o recebimento</t>
         </is>
       </c>
       <c r="G290" s="3" t="inlineStr">
         <is>
-          <t>Configuração</t>
+          <t>Ação</t>
         </is>
       </c>
       <c r="H290" s="3" t="inlineStr">
@@ -15604,22 +15604,22 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>Conferência do saldo com a Receita (CBS)</t>
+          <t>Previsão de entrada de caixa por tributo</t>
         </is>
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>Documento com saldo divergente na API de créditos da CBS sai do pedido e abre inconsistência. Evita pedir o que a Receita não reconhece.</t>
+          <t>Deferidos e em análise, datados pelo prazo legal, com correção estimada. Uma previsão para CBS e outra para IBS.</t>
         </is>
       </c>
       <c r="F291" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-12 Conferir com a Receita</t>
+          <t>PRD de Ressarcimento · F-10 Prever a entrada de caixa do tributo</t>
         </is>
       </c>
       <c r="G291" s="3" t="inlineStr">
         <is>
-          <t>Risco/Inc.</t>
+          <t>Analítico</t>
         </is>
       </c>
       <c r="H291" s="3" t="inlineStr">
@@ -15627,9 +15627,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I291" s="10" t="inlineStr">
-        <is>
-          <t>M1</t>
+      <c r="I291" s="9" t="inlineStr">
+        <is>
+          <t>M2</t>
         </is>
       </c>
       <c r="J291" s="3" t="inlineStr"/>
@@ -15655,22 +15655,22 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>Trilha de auditoria do pedido</t>
+          <t>Alertas de prazo do ressarcimento</t>
         </is>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>Quem declarou, aprovou, cancelou, registrou e decidiu, com data e valor, na linha do tempo de cada pedido.</t>
+          <t>Intenção, pedido, fim da análise e pagamento por silêncio, por tributo, na tela e como eventos da régua de Automações.</t>
         </is>
       </c>
       <c r="F292" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-13 Auditar</t>
+          <t>PRD de Ressarcimento · F-11 Alertar os prazos do tributo</t>
         </is>
       </c>
       <c r="G292" s="3" t="inlineStr">
         <is>
-          <t>Listagem</t>
+          <t>Configuração</t>
         </is>
       </c>
       <c r="H292" s="3" t="inlineStr">
@@ -15706,17 +15706,17 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>Impedimentos do IBS</t>
+          <t>Conferência do saldo com a Receita (CBS)</t>
         </is>
       </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>Auto de infração, cadastro irregular, notificação pendente ou débito exigível podem levar ao indeferimento do pedido de IBS. Aparece como alerta antes da intenção e do pedido.</t>
+          <t>Documento com saldo divergente na API de créditos da CBS sai do pedido e abre inconsistência. Evita pedir o que a Receita não reconhece.</t>
         </is>
       </c>
       <c r="F293" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-14 Verificar impedimentos do IBS</t>
+          <t>PRD de Ressarcimento · F-12 Conferir com a Receita</t>
         </is>
       </c>
       <c r="G293" s="3" t="inlineStr">
@@ -15757,22 +15757,22 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>Registrar o pedido de IBS (protocolo)</t>
+          <t>Trilha de auditoria do pedido</t>
         </is>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>Protocolo emitido pelo Comitê Gestor, data e valor. Acompanha o canal que o Comitê vier a definir.</t>
+          <t>Quem declarou, aprovou, cancelou, registrou e decidiu, com data e valor, na linha do tempo de cada pedido.</t>
         </is>
       </c>
       <c r="F294" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-15 Registrar o pedido de IBS</t>
+          <t>PRD de Ressarcimento · F-13 Auditar</t>
         </is>
       </c>
       <c r="G294" s="3" t="inlineStr">
         <is>
-          <t>Ação</t>
+          <t>Listagem</t>
         </is>
       </c>
       <c r="H294" s="3" t="inlineStr">
@@ -15792,13 +15792,115 @@
       <c r="N294" s="7" t="inlineStr"/>
       <c r="O294" s="8" t="inlineStr"/>
     </row>
+    <row r="295">
+      <c r="A295" s="3" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C295" s="3" t="inlineStr">
+        <is>
+          <t>Ressarcimento</t>
+        </is>
+      </c>
+      <c r="D295" s="4" t="inlineStr">
+        <is>
+          <t>Impedimentos do IBS</t>
+        </is>
+      </c>
+      <c r="E295" s="4" t="inlineStr">
+        <is>
+          <t>Auto de infração, cadastro irregular, notificação pendente ou débito exigível podem levar ao indeferimento do pedido de IBS. Aparece como alerta antes da intenção e do pedido.</t>
+        </is>
+      </c>
+      <c r="F295" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Ressarcimento · F-14 Verificar impedimentos do IBS</t>
+        </is>
+      </c>
+      <c r="G295" s="3" t="inlineStr">
+        <is>
+          <t>Risco/Inc.</t>
+        </is>
+      </c>
+      <c r="H295" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I295" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J295" s="3" t="inlineStr"/>
+      <c r="K295" s="3" t="inlineStr"/>
+      <c r="L295" s="3" t="inlineStr"/>
+      <c r="M295" s="7" t="inlineStr"/>
+      <c r="N295" s="7" t="inlineStr"/>
+      <c r="O295" s="8" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="3" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C296" s="3" t="inlineStr">
+        <is>
+          <t>Ressarcimento</t>
+        </is>
+      </c>
+      <c r="D296" s="4" t="inlineStr">
+        <is>
+          <t>Registrar o pedido de IBS (protocolo)</t>
+        </is>
+      </c>
+      <c r="E296" s="4" t="inlineStr">
+        <is>
+          <t>Protocolo emitido pelo Comitê Gestor, data e valor. Acompanha o canal que o Comitê vier a definir.</t>
+        </is>
+      </c>
+      <c r="F296" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Ressarcimento · F-15 Registrar o pedido de IBS</t>
+        </is>
+      </c>
+      <c r="G296" s="3" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="H296" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I296" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J296" s="3" t="inlineStr"/>
+      <c r="K296" s="3" t="inlineStr"/>
+      <c r="L296" s="3" t="inlineStr"/>
+      <c r="M296" s="7" t="inlineStr"/>
+      <c r="N296" s="7" t="inlineStr"/>
+      <c r="O296" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O294"/>
+  <autoFilter ref="A1:O296"/>
   <dataValidations count="2">
-    <dataValidation sqref="M2:M294" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use M0, M1, M2 ou Fora." promptTitle="Faixa revisada" prompt="Preencha apenas quando discordar da faixa proposta." type="list">
+    <dataValidation sqref="M2:M296" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use M0, M1, M2 ou Fora." promptTitle="Faixa revisada" prompt="Preencha apenas quando discordar da faixa proposta." type="list">
       <formula1>"M0,M1,M2,Fora"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N294" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Concorda com a faixa proposta?" prompt="Deixe em branco o que ainda não revisou." type="list">
+    <dataValidation sqref="N2:N296" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Concorda com a faixa proposta?" prompt="Deixe em branco o que ainda não revisou." type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16035,25 +16137,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F265" r:id="rId230"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F266" r:id="rId231"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F267" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F276" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F277" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F278" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F279" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F280" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F281" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F282" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F283" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F284" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F285" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F286" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F287" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F288" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F289" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F290" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F291" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F292" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F293" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F294" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F270" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F271" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F272" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F273" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F274" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F276" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F277" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F278" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F279" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F280" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F281" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F282" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F283" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F284" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F285" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F286" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F287" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F288" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F289" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F290" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F291" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F292" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F293" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F294" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F295" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F296" r:id="rId258"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16180,7 +16289,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>O módulo que a tese defende entra quase inteiro: 11 de 14. Ficam fora três gráficos analíticos — eles explicam o crédito, não o garantem. O Top 5 e Top 10 de fornecedores subiu na revisão de 15/09: saber de quem cobrar primeiro é operação, não análise. O painel Ressarcimento no ciclo do crédito entra em M1 (D17): o M0 do módulo não muda.</t>
+          <t>O módulo que a tese defende entra quase inteiro: 11 de 14. Ficam fora três gráficos analíticos — eles explicam o crédito, não o garantem. O Top 5 e Top 10 de fornecedores subiu na revisão de 15/09: saber de quem cobrar primeiro é operação, não análise. O painel Ressarcimento no ciclo do crédito entra em M1 (D17): o M0 do módulo não muda. A parcialidade (D19) passou ao mapa em 26/10, com o protótipo incorporado ao master: partição por tributo, selo por tributo, detalhe com as duas partições e histórico de movimentos, as quatro em M0.</t>
         </is>
       </c>
     </row>
@@ -16743,7 +16852,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>1</v>
@@ -16752,11 +16861,11 @@
         <v>0</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Multiusuário interno é consequência de adoção. A exceção é o painel de acessos externos, que entrou no M0 junto com o acesso do fornecedor — e foi confirmado na revisão de 15/09.</t>
+          <t>Multiusuário interno é consequência de adoção. A exceção é o painel de acessos externos, que entrou no M0 junto com o acesso do fornecedor — e foi confirmado na revisão de 15/09. A gestão de usuários implementada em 26/10 trouxe o histórico do usuário e a redefinição de senha pelo administrador, as duas em M1 com o resto do módulo. O que a autenticação muda no M0 está na D20, em aberto.</t>
         </is>
       </c>
     </row>
@@ -16802,7 +16911,7 @@
         <v>117</v>
       </c>
       <c r="D24" s="15" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E24" s="15" t="n">
         <v>35</v>
@@ -16811,7 +16920,7 @@
         <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -18097,7 +18206,7 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>v2.9</t>
+          <t>v2.10</t>
         </is>
       </c>
     </row>
@@ -18109,7 +18218,7 @@
       </c>
       <c r="B27" s="20" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
     </row>
@@ -18121,7 +18230,7 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Mapa de Funcionalidades v2.8</t>
+          <t>Mapa de Funcionalidades v2.9</t>
         </is>
       </c>
     </row>
@@ -18133,7 +18242,7 @@
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>293 funcionalidades · 21 módulos · 280 do mapa + 13 novas</t>
+          <t>295 funcionalidades · 21 módulos · 286 do mapa + 9 novas</t>
         </is>
       </c>
     </row>
@@ -18145,7 +18254,7 @@
       </c>
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>117 · 139 · 35 · 2</t>
+          <t>117 · 141 · 35 · 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(usuarios): escopo por CNPJ e decisoes finais da gestao de usuarios (R-250..R-254)
D-USR-05 A: convite e detalhe ganham o escopo (toda a organizacao ou
CNPJs por empresa); Administrador sempre com tudo; troca com motivo;
escopo parcial avisa que a apuracao da empresa fica de fora. D-USR-06 A:
troca de perfil so no prototipo. D-USR-07: sessao 30 min / 12 h.

Proposta v1.3 aprovada; PRD Organizacao v2.5; mapa v2.10 (entra o
escopo, sai a troca de perfil); priorizacao v2.11 com a D20 decidida:
login proprio em M0, SSO em M1, M0 em 116.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/docs/priorizacao-mvp.xlsx
+++ b/docs/docs/priorizacao-mvp.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Como revisar" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Priorização'!$A$1:$O$296</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Priorização'!$A$1:$O$297</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Revisões'!$A$1:$H$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O296"/>
+  <dimension ref="A1:O297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9064,12 +9064,12 @@
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>Após login, o usuário seleciona o perfil: Cliente (adquirente — acesso completo a todos os módulos) ou Fornecedor (acesso restrito ao portal com dados filtrados pelo CNPJ do fornecedor).</t>
-        </is>
-      </c>
-      <c r="F164" s="12" t="inlineStr">
-        <is>
-          <t>Sem PRD</t>
+          <t>Duas portas de entrada: quem é da organização entra com um dos quatro perfis internos, e o fornecedor entra no portal, restrito aos CNPJs do próprio acesso. O perfil vem do acesso de quem entrou, não de uma escolha na tela.</t>
+        </is>
+      </c>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G164" s="3" t="inlineStr">
@@ -9110,12 +9110,12 @@
       </c>
       <c r="D165" s="4" t="inlineStr">
         <is>
-          <t>Troca de perfil in-session</t>
+          <t>Tokens CSS globais + PALETTE JS</t>
         </is>
       </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
-          <t>Card do usuário no header e modal de configurações permitem alternar de perfil durante a sessão sem necessidade de novo login.</t>
+          <t>Todas as cores da interface definidas como variáveis CSS (--teal, --blue, --red etc.) e objeto PALETTE no JS. Nenhum valor hexadecimal inline no código — consistência visual garantida centralmente.</t>
         </is>
       </c>
       <c r="F165" s="12" t="inlineStr">
@@ -9125,7 +9125,7 @@
       </c>
       <c r="G165" s="3" t="inlineStr">
         <is>
-          <t>Ação</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="H165" s="3" t="inlineStr">
@@ -9161,12 +9161,12 @@
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>Tokens CSS globais + PALETTE JS</t>
+          <t>Sidebar teal colapsável + localStorage</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>Todas as cores da interface definidas como variáveis CSS (--teal, --blue, --red etc.) e objeto PALETTE no JS. Nenhum valor hexadecimal inline no código — consistência visual garantida centralmente.</t>
+          <t>Toggle de 56px com transição CSS suave entre expandida (labels visíveis) e colapsada (ícones com tooltips). Estado persistido em localStorage — mantido entre sessões e recarregamentos.</t>
         </is>
       </c>
       <c r="F166" s="12" t="inlineStr">
@@ -9212,12 +9212,12 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>Sidebar teal colapsável + localStorage</t>
+          <t>Tema claro/escuro automático</t>
         </is>
       </c>
       <c r="E167" s="4" t="inlineStr">
         <is>
-          <t>Toggle de 56px com transição CSS suave entre expandida (labels visíveis) e colapsada (ícones com tooltips). Estado persistido em localStorage — mantido entre sessões e recarregamentos.</t>
+          <t>prefers-color-scheme detecta o tema do sistema operacional e aplica automaticamente. Override manual disponível via atributo data-theme. Tokens redefinidos para cada tema sem hardcode de cores.</t>
         </is>
       </c>
       <c r="F167" s="12" t="inlineStr">
@@ -9263,12 +9263,12 @@
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>Tema claro/escuro automático</t>
+          <t>shBuildFilterPanel — filtros padronizados</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>prefers-color-scheme detecta o tema do sistema operacional e aplica automaticamente. Override manual disponível via atributo data-theme. Tokens redefinidos para cada tema sem hardcode de cores.</t>
+          <t>Função geradora de painéis de filtro colapsáveis com design unificado (classe sh-fp). Aplicada em Créditos, Débitos, Pagamentos, Inconsistências, Contratos, Fornecedores, Organização e Portal Fornecedor.</t>
         </is>
       </c>
       <c r="F168" s="12" t="inlineStr">
@@ -9314,12 +9314,12 @@
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>shBuildFilterPanel — filtros padronizados</t>
+          <t>RF Core — 10 colunas uniformes</t>
         </is>
       </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
-          <t>Função geradora de painéis de filtro colapsáveis com design unificado (classe sh-fp). Aplicada em Créditos, Débitos, Pagamentos, Inconsistências, Contratos, Fornecedores, Organização e Portal Fornecedor.</t>
+          <t>Conjunto padronizado de colunas presente em todas as listagens de RF do sistema: ID RF, Tipo Fiscal, DF Vinculado, Entidade, Data, Valor, Status do Crédito, Status de Registro, Método de Pagamento e Extinção. Filtros obrigatórios em todas as colunas.</t>
         </is>
       </c>
       <c r="F169" s="12" t="inlineStr">
@@ -9365,12 +9365,12 @@
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>RF Core — 10 colunas uniformes</t>
+          <t>ESC fecha qualquer modal</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>Conjunto padronizado de colunas presente em todas as listagens de RF do sistema: ID RF, Tipo Fiscal, DF Vinculado, Entidade, Data, Valor, Status do Crédito, Status de Registro, Método de Pagamento e Extinção. Filtros obrigatórios em todas as colunas.</t>
+          <t>Atalho de teclado global — qualquer overlay aberto no sistema (modais de detalhe NF, RF, inconsistência, fornecedor, contrato) responde ao ESC e fecha sem ação adicional do usuário.</t>
         </is>
       </c>
       <c r="F170" s="12" t="inlineStr">
@@ -9416,12 +9416,12 @@
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>ESC fecha qualquer modal</t>
+          <t>Tooltip de coluna como padrão de projeto</t>
         </is>
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t>Atalho de teclado global — qualquer overlay aberto no sistema (modais de detalhe NF, RF, inconsistência, fornecedor, contrato) responde ao ESC e fecha sem ação adicional do usuário.</t>
+          <t>Toda coluna declarada no catálogo de tabelas ganha explicação no cabeçalho, aplicada sempre do mesmo jeito. 104 colunas documentadas nas nove listagens; coluna nova só é publicada se souber se explicar.</t>
         </is>
       </c>
       <c r="F171" s="12" t="inlineStr">
@@ -9439,9 +9439,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I171" s="6" t="inlineStr">
-        <is>
-          <t>M0</t>
+      <c r="I171" s="13" t="inlineStr">
+        <is>
+          <t>Fora</t>
         </is>
       </c>
       <c r="J171" s="3" t="inlineStr"/>
@@ -9467,12 +9467,12 @@
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t>Tooltip de coluna como padrão de projeto</t>
+          <t>Documentação de produto dentro da aplicação</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>Toda coluna declarada no catálogo de tabelas ganha explicação no cabeçalho, aplicada sempre do mesmo jeito. 104 colunas documentadas nas nove listagens; coluna nova só é publicada se souber se explicar.</t>
+          <t>Hub de PRDs, mapa de funcionalidades e changelog acessíveis pela própria aplicação, sem depender de link externo. Quem opera e quem especifica leem a mesma versão.</t>
         </is>
       </c>
       <c r="F172" s="12" t="inlineStr">
@@ -9518,17 +9518,17 @@
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>Documentação de produto dentro da aplicação</t>
+          <t>Rotas diretas para telas e abas</t>
         </is>
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t>Hub de PRDs, mapa de funcionalidades e changelog acessíveis pela própria aplicação, sem depender de link externo. Quem opera e quem especifica leem a mesma versão.</t>
-        </is>
-      </c>
-      <c r="F173" s="12" t="inlineStr">
-        <is>
-          <t>Sem PRD</t>
+          <t>Endereços próprios para cada tela e aba, de forma que um link leve direto ao ponto certo da aplicação — usado em documentação, no hub de PRDs e no compartilhamento entre pessoas.</t>
+        </is>
+      </c>
+      <c r="F173" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Início · Seção 01 Contexto e posicionamento</t>
         </is>
       </c>
       <c r="G173" s="3" t="inlineStr">
@@ -9541,9 +9541,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I173" s="13" t="inlineStr">
-        <is>
-          <t>Fora</t>
+      <c r="I173" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
         </is>
       </c>
       <c r="J173" s="3" t="inlineStr"/>
@@ -9569,17 +9569,17 @@
       </c>
       <c r="D174" s="4" t="inlineStr">
         <is>
-          <t>Rotas diretas para telas e abas</t>
+          <t>Contador de filtros ativos sempre visível</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>Endereços próprios para cada tela e aba, de forma que um link leve direto ao ponto certo da aplicação — usado em documentação, no hub de PRDs e no compartilhamento entre pessoas.</t>
+          <t>Número filtrado nunca se confunde com total. Um indicador sob filtro, sem sinal de filtro, é erro de leitura esperando acontecer.</t>
         </is>
       </c>
       <c r="F174" s="5" t="inlineStr">
         <is>
-          <t>PRD de Início · Seção 01 Contexto e posicionamento</t>
+          <t>PRD de Arcabouço de interface · Seção 02 Painel de filtros</t>
         </is>
       </c>
       <c r="G174" s="3" t="inlineStr">
@@ -9620,12 +9620,12 @@
       </c>
       <c r="D175" s="4" t="inlineStr">
         <is>
-          <t>Contador de filtros ativos sempre visível</t>
+          <t>Filtro aplicado só sob confirmação</t>
         </is>
       </c>
       <c r="E175" s="4" t="inlineStr">
         <is>
-          <t>Número filtrado nunca se confunde com total. Um indicador sob filtro, sem sinal de filtro, é erro de leitura esperando acontecer.</t>
+          <t>O recorte inteiro é montado antes de a listagem ser refeita, em vez de recarregar a cada campo alterado.</t>
         </is>
       </c>
       <c r="F175" s="5" t="inlineStr">
@@ -9643,9 +9643,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I175" s="10" t="inlineStr">
-        <is>
-          <t>M1</t>
+      <c r="I175" s="9" t="inlineStr">
+        <is>
+          <t>M2</t>
         </is>
       </c>
       <c r="J175" s="3" t="inlineStr"/>
@@ -9671,17 +9671,17 @@
       </c>
       <c r="D176" s="4" t="inlineStr">
         <is>
-          <t>Filtro aplicado só sob confirmação</t>
+          <t>Paginação com retorno à primeira página</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>O recorte inteiro é montado antes de a listagem ser refeita, em vez de recarregar a cada campo alterado.</t>
+          <t>Mudar o recorte devolve a listagem ao início, para não mostrar a página 5 de um conjunto que acabou de mudar.</t>
         </is>
       </c>
       <c r="F176" s="5" t="inlineStr">
         <is>
-          <t>PRD de Arcabouço de interface · Seção 02 Painel de filtros</t>
+          <t>PRD de Arcabouço de interface · Seção 03 Pagina&amp;ccedil;&amp;atilde;o e busca</t>
         </is>
       </c>
       <c r="G176" s="3" t="inlineStr">
@@ -9722,12 +9722,12 @@
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>Paginação com retorno à primeira página</t>
+          <t>Alcance da busca declarado por módulo</t>
         </is>
       </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
-          <t>Mudar o recorte devolve a listagem ao início, para não mostrar a página 5 de um conjunto que acabou de mudar.</t>
+          <t>Cada módulo diz quais identificadores a própria busca encontra. Sem essa declaração, ninguém nota o que a busca deixou de fora.</t>
         </is>
       </c>
       <c r="F177" s="5" t="inlineStr">
@@ -9745,9 +9745,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I177" s="9" t="inlineStr">
-        <is>
-          <t>M2</t>
+      <c r="I177" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
         </is>
       </c>
       <c r="J177" s="3" t="inlineStr"/>
@@ -9773,17 +9773,17 @@
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>Alcance da busca declarado por módulo</t>
+          <t>Gerenciador de colunas com persistência por usuário</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>Cada módulo diz quais identificadores a própria busca encontra. Sem essa declaração, ninguém nota o que a busca deixou de fora.</t>
+          <t>Seleção, ordem e restauração do padrão, por listagem e por usuário, valendo também para a exportação.</t>
         </is>
       </c>
       <c r="F178" s="5" t="inlineStr">
         <is>
-          <t>PRD de Arcabouço de interface · Seção 03 Pagina&amp;ccedil;&amp;atilde;o e busca</t>
+          <t>PRD de Arcabouço de interface · Seção 04 Gerenciador de colunas</t>
         </is>
       </c>
       <c r="G178" s="3" t="inlineStr">
@@ -9796,9 +9796,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I178" s="10" t="inlineStr">
-        <is>
-          <t>M1</t>
+      <c r="I178" s="9" t="inlineStr">
+        <is>
+          <t>M2</t>
         </is>
       </c>
       <c r="J178" s="3" t="inlineStr"/>
@@ -9824,32 +9824,32 @@
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>Gerenciador de colunas com persistência por usuário</t>
+          <t>Login próprio por e-mail e senha</t>
         </is>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>Seleção, ordem e restauração do padrão, por listagem e por usuário, valendo também para a exportação.</t>
+          <t>E-mail e senha da própria pessoa, em provedor de identidade gerenciado, com convite, primeiro acesso, recuperação de senha, sessão de 30 minutos sem uso e trilha de entrada. Não existe no produto: hoje o acesso é uma senha no código. Entrou no MVP pela D20, no lugar do SSO.</t>
         </is>
       </c>
       <c r="F179" s="5" t="inlineStr">
         <is>
-          <t>PRD de Arcabouço de interface · Seção 04 Gerenciador de colunas</t>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G179" s="3" t="inlineStr">
         <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="H179" s="3" t="inlineStr">
-        <is>
-          <t>Mapa</t>
-        </is>
-      </c>
-      <c r="I179" s="9" t="inlineStr">
-        <is>
-          <t>M2</t>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="H179" s="11" t="inlineStr">
+        <is>
+          <t>Nova</t>
+        </is>
+      </c>
+      <c r="I179" s="6" t="inlineStr">
+        <is>
+          <t>M0</t>
         </is>
       </c>
       <c r="J179" s="3" t="inlineStr"/>
@@ -9880,12 +9880,12 @@
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>Entrada pelo provedor de identidade da empresa (SAML 2.0 ou OIDC), com provisionamento e revogação vindos de lá. Não existe no produto: hoje o acesso é uma senha no código.</t>
-        </is>
-      </c>
-      <c r="F180" s="12" t="inlineStr">
-        <is>
-          <t>Sem PRD</t>
+          <t>Entrada pelo provedor de identidade da empresa (SAML 2.0 ou OIDC), com provisionamento e revogação vindos de lá pelo SCIM. Fase 2 da gestão de usuários (D-USR-08); desceu do M0 pela D20.</t>
+        </is>
+      </c>
+      <c r="F180" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G180" s="3" t="inlineStr">
@@ -9898,9 +9898,9 @@
           <t>Nova</t>
         </is>
       </c>
-      <c r="I180" s="6" t="inlineStr">
-        <is>
-          <t>M0</t>
+      <c r="I180" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
         </is>
       </c>
       <c r="J180" s="3" t="inlineStr"/>
@@ -15135,32 +15135,32 @@
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>Operacional</t>
+          <t>Gestão</t>
         </is>
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>Ressarcimento</t>
+          <t>Usuários e Acessos</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>Saldo credor por período e tributo</t>
+          <t>Escopo por CNPJ do usuário</t>
         </is>
       </c>
       <c r="E282" s="4" t="inlineStr">
         <is>
-          <t>Por período e por tributo, na matriz: saldo inicial, apropriado, compensado, saldo credor, o que saiu para ressarcimento e o transportado. É a base da decisão de compensar ou pedir o dinheiro.</t>
+          <t>Cada usuário vê toda a organização ou só os CNPJs selecionados, e o Administrador vê sempre tudo. A troca é do administrador, com motivo, e fica na trilha. Quem tem só parte de uma empresa não vê a apuração nem o saldo dela, que são da empresa inteira. No protótipo o escopo é atribuído e registrado; o recorte das telas vem com o login de verdade.</t>
         </is>
       </c>
       <c r="F282" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-01 Ver o saldo credor do tributo</t>
+          <t>PRD de Organização · Seção 15 Usu&amp;aacute;rios e acessos</t>
         </is>
       </c>
       <c r="G282" s="3" t="inlineStr">
         <is>
-          <t>Listagem</t>
+          <t>Configuração</t>
         </is>
       </c>
       <c r="H282" s="3" t="inlineStr">
@@ -15196,22 +15196,22 @@
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>Comparar compensar e ressarcir</t>
+          <t>Saldo credor por período e tributo</t>
         </is>
       </c>
       <c r="E283" s="4" t="inlineStr">
         <is>
-          <t>Para o período em curso, as duas hipóteses lado a lado: uso do saldo, quando o dinheiro volta e a correção estimada pela Selic.</t>
+          <t>Por período e por tributo, na matriz: saldo inicial, apropriado, compensado, saldo credor, o que saiu para ressarcimento e o transportado. É a base da decisão de compensar ou pedir o dinheiro.</t>
         </is>
       </c>
       <c r="F283" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-02 Comparar compensar e ressarcir</t>
+          <t>PRD de Ressarcimento · F-01 Ver o saldo credor do tributo</t>
         </is>
       </c>
       <c r="G283" s="3" t="inlineStr">
         <is>
-          <t>Analítico</t>
+          <t>Listagem</t>
         </is>
       </c>
       <c r="H283" s="3" t="inlineStr">
@@ -15219,9 +15219,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I283" s="9" t="inlineStr">
-        <is>
-          <t>M2</t>
+      <c r="I283" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
         </is>
       </c>
       <c r="J283" s="3" t="inlineStr"/>
@@ -15247,22 +15247,22 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>Declarar e cancelar a intenção</t>
+          <t>Comparar compensar e ressarcir</t>
         </is>
       </c>
       <c r="E284" s="4" t="inlineStr">
         <is>
-          <t>Intenção do tributo até o último dia útil do período, com o efeito mostrado antes e aprovação acima do limite. Reserva o saldo; cancelada ou vencida, o saldo volta a compensar.</t>
+          <t>Para o período em curso, as duas hipóteses lado a lado: uso do saldo, quando o dinheiro volta e a correção estimada pela Selic.</t>
         </is>
       </c>
       <c r="F284" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-03 Declarar e cancelar a intenção</t>
+          <t>PRD de Ressarcimento · F-02 Comparar compensar e ressarcir</t>
         </is>
       </c>
       <c r="G284" s="3" t="inlineStr">
         <is>
-          <t>Ação</t>
+          <t>Analítico</t>
         </is>
       </c>
       <c r="H284" s="3" t="inlineStr">
@@ -15270,9 +15270,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I284" s="10" t="inlineStr">
-        <is>
-          <t>M1</t>
+      <c r="I284" s="9" t="inlineStr">
+        <is>
+          <t>M2</t>
         </is>
       </c>
       <c r="J284" s="3" t="inlineStr"/>
@@ -15298,17 +15298,17 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>Montar o pedido de CBS por documento</t>
+          <t>Declarar e cancelar a intenção</t>
         </is>
       </c>
       <c r="E285" s="4" t="inlineStr">
         <is>
-          <t>Escolhe os documentos do saldo reservado que entram no pedido. O que fica de fora volta a compensar desde a data do pedido.</t>
+          <t>Intenção do tributo até o último dia útil do período, com o efeito mostrado antes e aprovação acima do limite. Reserva o saldo; cancelada ou vencida, o saldo volta a compensar.</t>
         </is>
       </c>
       <c r="F285" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-04 Montar o pedido de CBS</t>
+          <t>PRD de Ressarcimento · F-03 Declarar e cancelar a intenção</t>
         </is>
       </c>
       <c r="G285" s="3" t="inlineStr">
@@ -15349,17 +15349,17 @@
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>Registrar o pedido de CBS (PER/DCOMP)</t>
+          <t>Montar o pedido de CBS por documento</t>
         </is>
       </c>
       <c r="E286" s="4" t="inlineStr">
         <is>
-          <t>Número do PER/DCOMP e data de transmissão. Calcula o fim da análise e a data do pagamento por silêncio do Fisco.</t>
+          <t>Escolhe os documentos do saldo reservado que entram no pedido. O que fica de fora volta a compensar desde a data do pedido.</t>
         </is>
       </c>
       <c r="F286" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-05 Registrar o pedido de CBS</t>
+          <t>PRD de Ressarcimento · F-04 Montar o pedido de CBS</t>
         </is>
       </c>
       <c r="G286" s="3" t="inlineStr">
@@ -15400,22 +15400,22 @@
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>Listagem de pedidos do tributo</t>
+          <t>Registrar o pedido de CBS (PER/DCOMP)</t>
         </is>
       </c>
       <c r="E287" s="4" t="inlineStr">
         <is>
-          <t>Pedidos com identificador no órgão, valor, prazo, contagem regressiva, situação e valor deferido.</t>
+          <t>Número do PER/DCOMP e data de transmissão. Calcula o fim da análise e a data do pagamento por silêncio do Fisco.</t>
         </is>
       </c>
       <c r="F287" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-06 Listar os pedidos do tributo</t>
+          <t>PRD de Ressarcimento · F-05 Registrar o pedido de CBS</t>
         </is>
       </c>
       <c r="G287" s="3" t="inlineStr">
         <is>
-          <t>Listagem</t>
+          <t>Ação</t>
         </is>
       </c>
       <c r="H287" s="3" t="inlineStr">
@@ -15451,22 +15451,22 @@
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>Acompanhar análise e fiscalização</t>
+          <t>Listagem de pedidos do tributo</t>
         </is>
       </c>
       <c r="E288" s="4" t="inlineStr">
         <is>
-          <t>Fiscalização suspende o prazo e tem limite de 360 dias. Mostra quando o prazo do Fisco se esgota sem manifestação.</t>
+          <t>Pedidos com identificador no órgão, valor, prazo, contagem regressiva, situação e valor deferido.</t>
         </is>
       </c>
       <c r="F288" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-07 Acompanhar análise, exigência e fiscalização</t>
+          <t>PRD de Ressarcimento · F-06 Listar os pedidos do tributo</t>
         </is>
       </c>
       <c r="G288" s="3" t="inlineStr">
         <is>
-          <t>Risco/Inc.</t>
+          <t>Listagem</t>
         </is>
       </c>
       <c r="H288" s="3" t="inlineStr">
@@ -15502,22 +15502,22 @@
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>Registrar decisão e cancelamento</t>
+          <t>Acompanhar análise e fiscalização</t>
         </is>
       </c>
       <c r="E289" s="4" t="inlineStr">
         <is>
-          <t>Deferido, deferido parcial, indeferido ou cancelado, cada um devolvendo o remanescente à compensação a partir da data que a norma define.</t>
+          <t>Fiscalização suspende o prazo e tem limite de 360 dias. Mostra quando o prazo do Fisco se esgota sem manifestação.</t>
         </is>
       </c>
       <c r="F289" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-08 Registrar a decisão e o cancelamento</t>
+          <t>PRD de Ressarcimento · F-07 Acompanhar análise, exigência e fiscalização</t>
         </is>
       </c>
       <c r="G289" s="3" t="inlineStr">
         <is>
-          <t>Ação</t>
+          <t>Risco/Inc.</t>
         </is>
       </c>
       <c r="H289" s="3" t="inlineStr">
@@ -15553,17 +15553,17 @@
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>Conciliar o recebimento com Selic</t>
+          <t>Registrar decisão e cancelamento</t>
         </is>
       </c>
       <c r="E290" s="4" t="inlineStr">
         <is>
-          <t>Recebido contra deferido corrigido. Extingue os créditos do pedido com o método Ressarcimento, e só aqui o status do crédito muda.</t>
+          <t>Deferido, deferido parcial, indeferido ou cancelado, cada um devolvendo o remanescente à compensação a partir da data que a norma define.</t>
         </is>
       </c>
       <c r="F290" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-09 Conciliar o recebimento</t>
+          <t>PRD de Ressarcimento · F-08 Registrar a decisão e o cancelamento</t>
         </is>
       </c>
       <c r="G290" s="3" t="inlineStr">
@@ -15604,22 +15604,22 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>Previsão de entrada de caixa por tributo</t>
+          <t>Conciliar o recebimento com Selic</t>
         </is>
       </c>
       <c r="E291" s="4" t="inlineStr">
         <is>
-          <t>Deferidos e em análise, datados pelo prazo legal, com correção estimada. Uma previsão para CBS e outra para IBS.</t>
+          <t>Recebido contra deferido corrigido. Extingue os créditos do pedido com o método Ressarcimento, e só aqui o status do crédito muda.</t>
         </is>
       </c>
       <c r="F291" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-10 Prever a entrada de caixa do tributo</t>
+          <t>PRD de Ressarcimento · F-09 Conciliar o recebimento</t>
         </is>
       </c>
       <c r="G291" s="3" t="inlineStr">
         <is>
-          <t>Analítico</t>
+          <t>Ação</t>
         </is>
       </c>
       <c r="H291" s="3" t="inlineStr">
@@ -15627,9 +15627,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I291" s="9" t="inlineStr">
-        <is>
-          <t>M2</t>
+      <c r="I291" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
         </is>
       </c>
       <c r="J291" s="3" t="inlineStr"/>
@@ -15655,22 +15655,22 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>Alertas de prazo do ressarcimento</t>
+          <t>Previsão de entrada de caixa por tributo</t>
         </is>
       </c>
       <c r="E292" s="4" t="inlineStr">
         <is>
-          <t>Intenção, pedido, fim da análise e pagamento por silêncio, por tributo, na tela e como eventos da régua de Automações.</t>
+          <t>Deferidos e em análise, datados pelo prazo legal, com correção estimada. Uma previsão para CBS e outra para IBS.</t>
         </is>
       </c>
       <c r="F292" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-11 Alertar os prazos do tributo</t>
+          <t>PRD de Ressarcimento · F-10 Prever a entrada de caixa do tributo</t>
         </is>
       </c>
       <c r="G292" s="3" t="inlineStr">
         <is>
-          <t>Configuração</t>
+          <t>Analítico</t>
         </is>
       </c>
       <c r="H292" s="3" t="inlineStr">
@@ -15678,9 +15678,9 @@
           <t>Mapa</t>
         </is>
       </c>
-      <c r="I292" s="10" t="inlineStr">
-        <is>
-          <t>M1</t>
+      <c r="I292" s="9" t="inlineStr">
+        <is>
+          <t>M2</t>
         </is>
       </c>
       <c r="J292" s="3" t="inlineStr"/>
@@ -15706,22 +15706,22 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>Conferência do saldo com a Receita (CBS)</t>
+          <t>Alertas de prazo do ressarcimento</t>
         </is>
       </c>
       <c r="E293" s="4" t="inlineStr">
         <is>
-          <t>Documento com saldo divergente na API de créditos da CBS sai do pedido e abre inconsistência. Evita pedir o que a Receita não reconhece.</t>
+          <t>Intenção, pedido, fim da análise e pagamento por silêncio, por tributo, na tela e como eventos da régua de Automações.</t>
         </is>
       </c>
       <c r="F293" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-12 Conferir com a Receita</t>
+          <t>PRD de Ressarcimento · F-11 Alertar os prazos do tributo</t>
         </is>
       </c>
       <c r="G293" s="3" t="inlineStr">
         <is>
-          <t>Risco/Inc.</t>
+          <t>Configuração</t>
         </is>
       </c>
       <c r="H293" s="3" t="inlineStr">
@@ -15757,22 +15757,22 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>Trilha de auditoria do pedido</t>
+          <t>Conferência do saldo com a Receita (CBS)</t>
         </is>
       </c>
       <c r="E294" s="4" t="inlineStr">
         <is>
-          <t>Quem declarou, aprovou, cancelou, registrou e decidiu, com data e valor, na linha do tempo de cada pedido.</t>
+          <t>Documento com saldo divergente na API de créditos da CBS sai do pedido e abre inconsistência. Evita pedir o que a Receita não reconhece.</t>
         </is>
       </c>
       <c r="F294" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-13 Auditar</t>
+          <t>PRD de Ressarcimento · F-12 Conferir com a Receita</t>
         </is>
       </c>
       <c r="G294" s="3" t="inlineStr">
         <is>
-          <t>Listagem</t>
+          <t>Risco/Inc.</t>
         </is>
       </c>
       <c r="H294" s="3" t="inlineStr">
@@ -15808,22 +15808,22 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>Impedimentos do IBS</t>
+          <t>Trilha de auditoria do pedido</t>
         </is>
       </c>
       <c r="E295" s="4" t="inlineStr">
         <is>
-          <t>Auto de infração, cadastro irregular, notificação pendente ou débito exigível podem levar ao indeferimento do pedido de IBS. Aparece como alerta antes da intenção e do pedido.</t>
+          <t>Quem declarou, aprovou, cancelou, registrou e decidiu, com data e valor, na linha do tempo de cada pedido.</t>
         </is>
       </c>
       <c r="F295" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-14 Verificar impedimentos do IBS</t>
+          <t>PRD de Ressarcimento · F-13 Auditar</t>
         </is>
       </c>
       <c r="G295" s="3" t="inlineStr">
         <is>
-          <t>Risco/Inc.</t>
+          <t>Listagem</t>
         </is>
       </c>
       <c r="H295" s="3" t="inlineStr">
@@ -15859,22 +15859,22 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>Registrar o pedido de IBS (protocolo)</t>
+          <t>Impedimentos do IBS</t>
         </is>
       </c>
       <c r="E296" s="4" t="inlineStr">
         <is>
-          <t>Protocolo emitido pelo Comitê Gestor, data e valor. Acompanha o canal que o Comitê vier a definir.</t>
+          <t>Auto de infração, cadastro irregular, notificação pendente ou débito exigível podem levar ao indeferimento do pedido de IBS. Aparece como alerta antes da intenção e do pedido.</t>
         </is>
       </c>
       <c r="F296" s="5" t="inlineStr">
         <is>
-          <t>PRD de Ressarcimento · F-15 Registrar o pedido de IBS</t>
+          <t>PRD de Ressarcimento · F-14 Verificar impedimentos do IBS</t>
         </is>
       </c>
       <c r="G296" s="3" t="inlineStr">
         <is>
-          <t>Ação</t>
+          <t>Risco/Inc.</t>
         </is>
       </c>
       <c r="H296" s="3" t="inlineStr">
@@ -15894,13 +15894,64 @@
       <c r="N296" s="7" t="inlineStr"/>
       <c r="O296" s="8" t="inlineStr"/>
     </row>
+    <row r="297">
+      <c r="A297" s="3" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C297" s="3" t="inlineStr">
+        <is>
+          <t>Ressarcimento</t>
+        </is>
+      </c>
+      <c r="D297" s="4" t="inlineStr">
+        <is>
+          <t>Registrar o pedido de IBS (protocolo)</t>
+        </is>
+      </c>
+      <c r="E297" s="4" t="inlineStr">
+        <is>
+          <t>Protocolo emitido pelo Comitê Gestor, data e valor. Acompanha o canal que o Comitê vier a definir.</t>
+        </is>
+      </c>
+      <c r="F297" s="5" t="inlineStr">
+        <is>
+          <t>PRD de Ressarcimento · F-15 Registrar o pedido de IBS</t>
+        </is>
+      </c>
+      <c r="G297" s="3" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="H297" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I297" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J297" s="3" t="inlineStr"/>
+      <c r="K297" s="3" t="inlineStr"/>
+      <c r="L297" s="3" t="inlineStr"/>
+      <c r="M297" s="7" t="inlineStr"/>
+      <c r="N297" s="7" t="inlineStr"/>
+      <c r="O297" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O296"/>
+  <autoFilter ref="A1:O297"/>
   <dataValidations count="2">
-    <dataValidation sqref="M2:M296" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use M0, M1, M2 ou Fora." promptTitle="Faixa revisada" prompt="Preencha apenas quando discordar da faixa proposta." type="list">
+    <dataValidation sqref="M2:M297" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use M0, M1, M2 ou Fora." promptTitle="Faixa revisada" prompt="Preencha apenas quando discordar da faixa proposta." type="list">
       <formula1>"M0,M1,M2,Fora"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N296" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Concorda com a faixa proposta?" prompt="Deixe em branco o que ainda não revisou." type="list">
+    <dataValidation sqref="N2:N297" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Concorda com a faixa proposta?" prompt="Deixe em branco o que ainda não revisou." type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16055,114 +16106,118 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F158" r:id="rId148"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F159" r:id="rId149"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F160" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F178" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F182" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F183" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F185" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F187" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F188" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F189" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F190" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F191" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F192" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F193" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F194" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F195" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F196" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F197" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F205" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F206" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F207" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F208" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F209" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F210" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F211" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F212" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F213" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F214" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F215" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F216" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F217" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F218" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F219" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F220" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F221" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F222" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F227" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F228" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F229" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F230" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F231" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F232" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F233" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F234" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F235" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F243" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F244" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F245" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F246" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F247" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F248" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F249" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F250" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F251" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F252" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F253" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F254" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F255" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F256" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F257" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F258" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F259" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F260" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F261" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F262" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F263" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F264" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F265" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F266" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F267" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F270" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F271" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F272" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F273" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F274" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F276" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F277" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F278" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F279" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F280" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F281" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F282" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F283" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F284" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F285" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F286" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F287" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F288" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F289" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F290" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F291" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F292" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F293" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F294" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F295" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F296" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F173" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F178" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F180" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F182" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F183" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F185" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F187" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F188" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F189" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F190" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F191" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F192" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F193" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F194" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F195" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F196" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F197" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F205" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F206" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F207" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F208" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F209" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F210" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F211" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F212" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F213" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F214" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F215" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F216" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F217" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F218" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F219" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F220" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F221" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F222" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F227" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F228" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F229" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F230" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F231" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F232" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F233" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F234" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F235" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F243" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F244" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F245" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F246" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F247" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F248" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F249" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F250" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F251" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F252" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F253" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F254" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F255" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F256" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F257" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F258" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F259" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F260" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F261" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F262" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F263" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F264" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F265" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F266" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F267" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F270" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F271" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F272" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F273" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F274" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F276" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F277" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F278" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F279" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F280" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F281" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F282" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F283" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F284" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F285" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F286" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F287" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F288" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F289" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F290" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F291" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F292" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F293" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F294" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F295" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F296" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F297" r:id="rId262"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16625,10 +16680,10 @@
         </is>
       </c>
       <c r="C14" s="14" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>3</v>
@@ -16641,7 +16696,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Login, perfis e o sistema de design, mais o selo de modo demonstração da troca de perfil. O SSO corporativo continua sendo a única funcionalidade do MVP que não existe em parte alguma.</t>
+          <t>Login, perfis e o sistema de design. Pela D20, de 26/10, o MVP entra com o login próprio por e-mail e senha, que ainda não existe, e o SSO corporativo desce a M1, para a fase 2 com o SCIM. A troca de perfil saiu do inventário: é só do protótipo (D-USR-06).</t>
         </is>
       </c>
     </row>
@@ -16852,7 +16907,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>1</v>
@@ -16861,11 +16916,11 @@
         <v>0</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Multiusuário interno é consequência de adoção. A exceção é o painel de acessos externos, que entrou no M0 junto com o acesso do fornecedor — e foi confirmado na revisão de 15/09. A gestão de usuários implementada em 26/10 trouxe o histórico do usuário e a redefinição de senha pelo administrador, as duas em M1 com o resto do módulo. O que a autenticação muda no M0 está na D20, em aberto.</t>
+          <t>Multiusuário interno é consequência de adoção. A exceção é o painel de acessos externos, que entrou no M0 junto com o acesso do fornecedor — e foi confirmado na revisão de 15/09. A gestão de usuários implementada em 26/10 trouxe o histórico do usuário e a redefinição de senha pelo administrador, as duas em M1 com o resto do módulo. O escopo por CNPJ (D-USR-05) também entra em M1, pelo critério: é multiusuário, e a cadeia do crédito fecha sem ele. O que a autenticação muda no M0 está na D20.</t>
         </is>
       </c>
     </row>
@@ -16908,10 +16963,10 @@
         </is>
       </c>
       <c r="C24" s="15" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D24" s="15" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E24" s="15" t="n">
         <v>35</v>
@@ -16920,7 +16975,7 @@
         <v>2</v>
       </c>
       <c r="G24" s="15" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
   </sheetData>
@@ -18206,7 +18261,7 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>v2.10</t>
+          <t>v2.11</t>
         </is>
       </c>
     </row>
@@ -18230,7 +18285,7 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Mapa de Funcionalidades v2.9</t>
+          <t>Mapa de Funcionalidades v2.10</t>
         </is>
       </c>
     </row>
@@ -18242,7 +18297,7 @@
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>295 funcionalidades · 21 módulos · 286 do mapa + 9 novas</t>
+          <t>296 funcionalidades · 21 módulos · 286 do mapa + 10 novas</t>
         </is>
       </c>
     </row>
@@ -18254,7 +18309,7 @@
       </c>
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>117 · 141 · 35 · 2</t>
+          <t>116 · 143 · 35 · 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(pcont): PCONT no app; mapa v2.11, priorizacao v2.12, PRDs PCONT v1.2 e Apuracao v1.5 (R-277)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/docs/priorizacao-mvp.xlsx
+++ b/docs/docs/priorizacao-mvp.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Como revisar" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Priorização'!$A$1:$O$297</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Priorização'!$A$1:$O$317</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Revisões'!$A$1:$H$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O297"/>
+  <dimension ref="A1:O317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -15945,13 +15945,1033 @@
       <c r="N297" s="7" t="inlineStr"/>
       <c r="O297" s="8" t="inlineStr"/>
     </row>
+    <row r="298">
+      <c r="A298" s="3" t="n">
+        <v>297</v>
+      </c>
+      <c r="B298" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C298" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D298" s="4" t="inlineStr">
+        <is>
+          <t>Empresa do grupo econômico</t>
+        </is>
+      </c>
+      <c r="E298" s="4" t="inlineStr">
+        <is>
+          <t>Escolhe a empresa pelo CNPJ raiz, com a matriz que centraliza o recolhimento; competências, saldos, divergências, guias e histórico passam a ser dela.</t>
+        </is>
+      </c>
+      <c r="F298" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-01 Escolher a empresa do grupo</t>
+        </is>
+      </c>
+      <c r="G298" s="3" t="inlineStr">
+        <is>
+          <t>Configuração</t>
+        </is>
+      </c>
+      <c r="H298" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I298" s="6" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="J298" s="3" t="inlineStr"/>
+      <c r="K298" s="3" t="inlineStr"/>
+      <c r="L298" s="3" t="inlineStr"/>
+      <c r="M298" s="7" t="inlineStr"/>
+      <c r="N298" s="7" t="inlineStr"/>
+      <c r="O298" s="8" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="3" t="n">
+        <v>298</v>
+      </c>
+      <c r="B299" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C299" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D299" s="4" t="inlineStr">
+        <is>
+          <t>Competências com a etapa e o prazo do ente</t>
+        </is>
+      </c>
+      <c r="E299" s="4" t="inlineStr">
+        <is>
+          <t>Carrossel do exercício com a etapa de cada tributo na Receita Federal e no Comitê Gestor — em apuração, entrega, ajustes, vencimento — e os dias até o prazo.</t>
+        </is>
+      </c>
+      <c r="F299" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-02 Competências com a etapa e o prazo</t>
+        </is>
+      </c>
+      <c r="G299" s="3" t="inlineStr">
+        <is>
+          <t>Listagem</t>
+        </is>
+      </c>
+      <c r="H299" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I299" s="6" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="J299" s="3" t="inlineStr"/>
+      <c r="K299" s="3" t="inlineStr"/>
+      <c r="L299" s="3" t="inlineStr"/>
+      <c r="M299" s="7" t="inlineStr"/>
+      <c r="N299" s="7" t="inlineStr"/>
+      <c r="O299" s="8" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="3" t="n">
+        <v>299</v>
+      </c>
+      <c r="B300" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C300" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D300" s="4" t="inlineStr">
+        <is>
+          <t>Visão consolidada sem somar tributos</t>
+        </is>
+      </c>
+      <c r="E300" s="4" t="inlineStr">
+        <is>
+          <t>CBS e IBS lado a lado: saldo do SplitHub, saldo do ente, diferença, divergências e guia. Os saldos dos dois tributos nunca se somam.</t>
+        </is>
+      </c>
+      <c r="F300" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-03 Visão consolidada da competência</t>
+        </is>
+      </c>
+      <c r="G300" s="3" t="inlineStr">
+        <is>
+          <t>Analítico</t>
+        </is>
+      </c>
+      <c r="H300" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I300" s="6" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="J300" s="3" t="inlineStr"/>
+      <c r="K300" s="3" t="inlineStr"/>
+      <c r="L300" s="3" t="inlineStr"/>
+      <c r="M300" s="7" t="inlineStr"/>
+      <c r="N300" s="7" t="inlineStr"/>
+      <c r="O300" s="8" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="B301" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C301" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D301" s="4" t="inlineStr">
+        <is>
+          <t>Desembolso da competência</t>
+        </is>
+      </c>
+      <c r="E301" s="4" t="inlineStr">
+        <is>
+          <t>As duas guias do mês e o total de caixa, com os entes nomeados. É a visão da tesouraria; não é saldo e não entra em apuração.</t>
+        </is>
+      </c>
+      <c r="F301" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-04 Desembolso da competência</t>
+        </is>
+      </c>
+      <c r="G301" s="3" t="inlineStr">
+        <is>
+          <t>Analítico</t>
+        </is>
+      </c>
+      <c r="H301" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I301" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J301" s="3" t="inlineStr"/>
+      <c r="K301" s="3" t="inlineStr"/>
+      <c r="L301" s="3" t="inlineStr"/>
+      <c r="M301" s="7" t="inlineStr"/>
+      <c r="N301" s="7" t="inlineStr"/>
+      <c r="O301" s="8" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="3" t="n">
+        <v>301</v>
+      </c>
+      <c r="B302" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C302" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D302" s="4" t="inlineStr">
+        <is>
+          <t>Demonstrativo SplitHub × ente</t>
+        </is>
+      </c>
+      <c r="E302" s="4" t="inlineStr">
+        <is>
+          <t>As linhas do art. 44 com três colunas — SplitHub, ente e diferença —, o resultado antes do PCONT, o saldo atualizado e os créditos a apropriar.</t>
+        </is>
+      </c>
+      <c r="F302" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-05 Demonstrativo SplitHub × ente</t>
+        </is>
+      </c>
+      <c r="G302" s="3" t="inlineStr">
+        <is>
+          <t>Listagem</t>
+        </is>
+      </c>
+      <c r="H302" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I302" s="6" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="J302" s="3" t="inlineStr"/>
+      <c r="K302" s="3" t="inlineStr"/>
+      <c r="L302" s="3" t="inlineStr"/>
+      <c r="M302" s="7" t="inlineStr"/>
+      <c r="N302" s="7" t="inlineStr"/>
+      <c r="O302" s="8" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="3" t="n">
+        <v>302</v>
+      </c>
+      <c r="B303" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C303" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D303" s="4" t="inlineStr">
+        <is>
+          <t>Detalhamento até o conta corrente da operação</t>
+        </is>
+      </c>
+      <c r="E303" s="4" t="inlineStr">
+        <is>
+          <t>Linha, origem, documento por contraparte e o conta corrente da nota no SplitHub ao lado do ente, com busca, filtro de divergência e CSV.</t>
+        </is>
+      </c>
+      <c r="F303" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-06 Detalhamento até a nota</t>
+        </is>
+      </c>
+      <c r="G303" s="3" t="inlineStr">
+        <is>
+          <t>Listagem</t>
+        </is>
+      </c>
+      <c r="H303" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I303" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J303" s="3" t="inlineStr"/>
+      <c r="K303" s="3" t="inlineStr"/>
+      <c r="L303" s="3" t="inlineStr"/>
+      <c r="M303" s="7" t="inlineStr"/>
+      <c r="N303" s="7" t="inlineStr"/>
+      <c r="O303" s="8" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="3" t="n">
+        <v>303</v>
+      </c>
+      <c r="B304" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C304" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D304" s="4" t="inlineStr">
+        <is>
+          <t>Recalcular, fechar e reabrir por tributo</t>
+        </is>
+      </c>
+      <c r="E304" s="4" t="inlineStr">
+        <is>
+          <t>O ciclo que era da tela da Apuração IBS/CBS, agora por tributo: recalcular a partir dos documentos, fechar com justificativa quando há divergência e reabrir.</t>
+        </is>
+      </c>
+      <c r="F304" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-07 Recalcular, fechar e reabrir</t>
+        </is>
+      </c>
+      <c r="G304" s="3" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="H304" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I304" s="6" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="J304" s="3" t="inlineStr"/>
+      <c r="K304" s="3" t="inlineStr"/>
+      <c r="L304" s="3" t="inlineStr"/>
+      <c r="M304" s="7" t="inlineStr"/>
+      <c r="N304" s="7" t="inlineStr"/>
+      <c r="O304" s="8" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="3" t="n">
+        <v>304</v>
+      </c>
+      <c r="B305" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C305" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D305" s="4" t="inlineStr">
+        <is>
+          <t>Linha do tempo da competência por ente</t>
+        </is>
+      </c>
+      <c r="E305" s="4" t="inlineStr">
+        <is>
+          <t>Trilhos da Receita Federal e do Comitê Gestor e as etapas E1 a E8, da apuração do mês à extinção, com o que aconteceu em cada uma.</t>
+        </is>
+      </c>
+      <c r="F305" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-08 Linha do tempo por ente</t>
+        </is>
+      </c>
+      <c r="G305" s="3" t="inlineStr">
+        <is>
+          <t>Listagem</t>
+        </is>
+      </c>
+      <c r="H305" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I305" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J305" s="3" t="inlineStr"/>
+      <c r="K305" s="3" t="inlineStr"/>
+      <c r="L305" s="3" t="inlineStr"/>
+      <c r="M305" s="7" t="inlineStr"/>
+      <c r="N305" s="7" t="inlineStr"/>
+      <c r="O305" s="8" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="3" t="n">
+        <v>305</v>
+      </c>
+      <c r="B306" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C306" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D306" s="4" t="inlineStr">
+        <is>
+          <t>Divergências por tributo e natureza, com chamado</t>
+        </is>
+      </c>
+      <c r="E306" s="4" t="inlineStr">
+        <is>
+          <t>Toda diferença num documento abre chamado sozinha. Lista com valores, efeito no saldo do ente e tipo do catálogo, filtrada por tributo e por crédito ou débito.</t>
+        </is>
+      </c>
+      <c r="F306" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-09 Divergências por tributo e natureza</t>
+        </is>
+      </c>
+      <c r="G306" s="3" t="inlineStr">
+        <is>
+          <t>Risco/Inc.</t>
+        </is>
+      </c>
+      <c r="H306" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I306" s="6" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="J306" s="3" t="inlineStr"/>
+      <c r="K306" s="3" t="inlineStr"/>
+      <c r="L306" s="3" t="inlineStr"/>
+      <c r="M306" s="7" t="inlineStr"/>
+      <c r="N306" s="7" t="inlineStr"/>
+      <c r="O306" s="8" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="3" t="n">
+        <v>306</v>
+      </c>
+      <c r="B307" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C307" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D307" s="4" t="inlineStr">
+        <is>
+          <t>Decisão registrada por divergência</t>
+        </is>
+      </c>
+      <c r="E307" s="4" t="inlineStr">
+        <is>
+          <t>Aguardar o reflexo, aceitar, ajustar no portal, importar ou corrigir, com quem e quando. O ajuste entra no valor sugerido da guia; emitir sem decidir pede justificativa.</t>
+        </is>
+      </c>
+      <c r="F307" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-10 Decisão por divergência</t>
+        </is>
+      </c>
+      <c r="G307" s="3" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="H307" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I307" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J307" s="3" t="inlineStr"/>
+      <c r="K307" s="3" t="inlineStr"/>
+      <c r="L307" s="3" t="inlineStr"/>
+      <c r="M307" s="7" t="inlineStr"/>
+      <c r="N307" s="7" t="inlineStr"/>
+      <c r="O307" s="8" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="3" t="n">
+        <v>307</v>
+      </c>
+      <c r="B308" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C308" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D308" s="4" t="inlineStr">
+        <is>
+          <t>Emissão do DARF da CBS</t>
+        </is>
+      </c>
+      <c r="E308" s="4" t="inlineStr">
+        <is>
+          <t>Guia do saldo pela Receita Federal, no valor do ente após os ajustes, do SplitHub ou outro. A emissão por API foi anunciada pela Receita, ainda sem documentação.</t>
+        </is>
+      </c>
+      <c r="F308" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-11 Emitir o DARF da CBS</t>
+        </is>
+      </c>
+      <c r="G308" s="3" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="H308" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I308" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J308" s="3" t="inlineStr"/>
+      <c r="K308" s="3" t="inlineStr"/>
+      <c r="L308" s="3" t="inlineStr"/>
+      <c r="M308" s="7" t="inlineStr"/>
+      <c r="N308" s="7" t="inlineStr"/>
+      <c r="O308" s="8" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="3" t="n">
+        <v>308</v>
+      </c>
+      <c r="B309" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C309" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D309" s="4" t="inlineStr">
+        <is>
+          <t>Guia do IBS registrada do portal</t>
+        </is>
+      </c>
+      <c r="E309" s="4" t="inlineStr">
+        <is>
+          <t>Enquanto o Comitê Gestor não emite por API, a guia do portal entra com linha digitável, valor e PDF, e o resto do fluxo funciona igual.</t>
+        </is>
+      </c>
+      <c r="F309" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-12 Registrar a guia do IBS do portal</t>
+        </is>
+      </c>
+      <c r="G309" s="3" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="H309" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I309" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J309" s="3" t="inlineStr"/>
+      <c r="K309" s="3" t="inlineStr"/>
+      <c r="L309" s="3" t="inlineStr"/>
+      <c r="M309" s="7" t="inlineStr"/>
+      <c r="N309" s="7" t="inlineStr"/>
+      <c r="O309" s="8" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="3" t="n">
+        <v>309</v>
+      </c>
+      <c r="B310" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C310" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D310" s="4" t="inlineStr">
+        <is>
+          <t>Simulação de pagamento parcial</t>
+        </is>
+      </c>
+      <c r="E310" s="4" t="inlineStr">
+        <is>
+          <t>Quantas notas um valor extingue na ordem cronológica e quais clientes ficam sem crédito. Explica o efeito de pagar menos antes de pagar.</t>
+        </is>
+      </c>
+      <c r="F310" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-13 Simular o pagamento parcial</t>
+        </is>
+      </c>
+      <c r="G310" s="3" t="inlineStr">
+        <is>
+          <t>Analítico</t>
+        </is>
+      </c>
+      <c r="H310" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I310" s="9" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="J310" s="3" t="inlineStr"/>
+      <c r="K310" s="3" t="inlineStr"/>
+      <c r="L310" s="3" t="inlineStr"/>
+      <c r="M310" s="7" t="inlineStr"/>
+      <c r="N310" s="7" t="inlineStr"/>
+      <c r="O310" s="8" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="3" t="n">
+        <v>310</v>
+      </c>
+      <c r="B311" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C311" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D311" s="4" t="inlineStr">
+        <is>
+          <t>Envio ao ERP e comprovante de volta</t>
+        </is>
+      </c>
+      <c r="E311" s="4" t="inlineStr">
+        <is>
+          <t>pcont.guide_issued leva a guia, a apuração do mês e a decomposição; o comprovante volta por POST /v1/pcont/proofs.</t>
+        </is>
+      </c>
+      <c r="F311" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-14 Enviar ao ERP e receber o comprovante</t>
+        </is>
+      </c>
+      <c r="G311" s="3" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="H311" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I311" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J311" s="3" t="inlineStr"/>
+      <c r="K311" s="3" t="inlineStr"/>
+      <c r="L311" s="3" t="inlineStr"/>
+      <c r="M311" s="7" t="inlineStr"/>
+      <c r="N311" s="7" t="inlineStr"/>
+      <c r="O311" s="8" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="3" t="n">
+        <v>311</v>
+      </c>
+      <c r="B312" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C312" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D312" s="4" t="inlineStr">
+        <is>
+          <t>Acompanhamento até a extinção</t>
+        </is>
+      </c>
+      <c r="E312" s="4" t="inlineStr">
+        <is>
+          <t>Processamento pelo ente com as notas extintas e os clientes liberados; cancelar, substituir quando o saldo muda e emitir a guia do restante.</t>
+        </is>
+      </c>
+      <c r="F312" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-15 Acompanhar até a extinção</t>
+        </is>
+      </c>
+      <c r="G312" s="3" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="H312" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I312" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J312" s="3" t="inlineStr"/>
+      <c r="K312" s="3" t="inlineStr"/>
+      <c r="L312" s="3" t="inlineStr"/>
+      <c r="M312" s="7" t="inlineStr"/>
+      <c r="N312" s="7" t="inlineStr"/>
+      <c r="O312" s="8" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="3" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C313" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D313" s="4" t="inlineStr">
+        <is>
+          <t>Encargos simulados de atraso</t>
+        </is>
+      </c>
+      <c r="E313" s="4" t="inlineStr">
+        <is>
+          <t>Multa e juros quando a guia passa do vencimento sem pagamento, simulados como no RAD.</t>
+        </is>
+      </c>
+      <c r="F313" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-16 Encargos simulados de atraso</t>
+        </is>
+      </c>
+      <c r="G313" s="3" t="inlineStr">
+        <is>
+          <t>Analítico</t>
+        </is>
+      </c>
+      <c r="H313" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I313" s="9" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="J313" s="3" t="inlineStr"/>
+      <c r="K313" s="3" t="inlineStr"/>
+      <c r="L313" s="3" t="inlineStr"/>
+      <c r="M313" s="7" t="inlineStr"/>
+      <c r="N313" s="7" t="inlineStr"/>
+      <c r="O313" s="8" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="3" t="n">
+        <v>313</v>
+      </c>
+      <c r="B314" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C314" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D314" s="4" t="inlineStr">
+        <is>
+          <t>Histórico com retrato do demonstrativo</t>
+        </is>
+      </c>
+      <c r="E314" s="4" t="inlineStr">
+        <is>
+          <t>Guias por tributo e competência, com a linha do tempo e o demonstrativo congelado na emissão, mesmo que o ente mude depois.</t>
+        </is>
+      </c>
+      <c r="F314" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-17 Histórico com retrato</t>
+        </is>
+      </c>
+      <c r="G314" s="3" t="inlineStr">
+        <is>
+          <t>Listagem</t>
+        </is>
+      </c>
+      <c r="H314" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I314" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J314" s="3" t="inlineStr"/>
+      <c r="K314" s="3" t="inlineStr"/>
+      <c r="L314" s="3" t="inlineStr"/>
+      <c r="M314" s="7" t="inlineStr"/>
+      <c r="N314" s="7" t="inlineStr"/>
+      <c r="O314" s="8" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="3" t="n">
+        <v>314</v>
+      </c>
+      <c r="B315" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C315" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D315" s="4" t="inlineStr">
+        <is>
+          <t>Exportação do demonstrativo</t>
+        </is>
+      </c>
+      <c r="E315" s="4" t="inlineStr">
+        <is>
+          <t>CSV do tributo ou da competência, e do detalhamento por documento.</t>
+        </is>
+      </c>
+      <c r="F315" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-18 Exportar</t>
+        </is>
+      </c>
+      <c r="G315" s="3" t="inlineStr">
+        <is>
+          <t>Ação</t>
+        </is>
+      </c>
+      <c r="H315" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I315" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J315" s="3" t="inlineStr"/>
+      <c r="K315" s="3" t="inlineStr"/>
+      <c r="L315" s="3" t="inlineStr"/>
+      <c r="M315" s="7" t="inlineStr"/>
+      <c r="N315" s="7" t="inlineStr"/>
+      <c r="O315" s="8" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="3" t="n">
+        <v>315</v>
+      </c>
+      <c r="B316" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C316" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D316" s="4" t="inlineStr">
+        <is>
+          <t>Painel executivo do grupo econômico</t>
+        </is>
+      </c>
+      <c r="E316" s="4" t="inlineStr">
+        <is>
+          <t>Grupo ou empresa por competência: indicadores por tributo, alertas, tabela das empresas, saldo por mês, composição, mapa de etapas e funil das guias.</t>
+        </is>
+      </c>
+      <c r="F316" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-19 Painel executivo do grupo</t>
+        </is>
+      </c>
+      <c r="G316" s="3" t="inlineStr">
+        <is>
+          <t>Analítico</t>
+        </is>
+      </c>
+      <c r="H316" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I316" s="9" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="J316" s="3" t="inlineStr"/>
+      <c r="K316" s="3" t="inlineStr"/>
+      <c r="L316" s="3" t="inlineStr"/>
+      <c r="M316" s="7" t="inlineStr"/>
+      <c r="N316" s="7" t="inlineStr"/>
+      <c r="O316" s="8" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="3" t="n">
+        <v>316</v>
+      </c>
+      <c r="B317" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="C317" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="D317" s="4" t="inlineStr">
+        <is>
+          <t>Auditoria das ações</t>
+        </is>
+      </c>
+      <c r="E317" s="4" t="inlineStr">
+        <is>
+          <t>Trilha encadeada por hash de tudo que muda o estado do módulo — tela, API e sistema —, com quem, antes e depois e motivo; filtros, integridade e CSV.</t>
+        </is>
+      </c>
+      <c r="F317" s="5" t="inlineStr">
+        <is>
+          <t>PRD de PCONT · F-20 Auditoria das ações</t>
+        </is>
+      </c>
+      <c r="G317" s="3" t="inlineStr">
+        <is>
+          <t>Listagem</t>
+        </is>
+      </c>
+      <c r="H317" s="3" t="inlineStr">
+        <is>
+          <t>Mapa</t>
+        </is>
+      </c>
+      <c r="I317" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="J317" s="3" t="inlineStr"/>
+      <c r="K317" s="3" t="inlineStr"/>
+      <c r="L317" s="3" t="inlineStr"/>
+      <c r="M317" s="7" t="inlineStr"/>
+      <c r="N317" s="7" t="inlineStr"/>
+      <c r="O317" s="8" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O297"/>
+  <autoFilter ref="A1:O317"/>
   <dataValidations count="2">
-    <dataValidation sqref="M2:M297" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use M0, M1, M2 ou Fora." promptTitle="Faixa revisada" prompt="Preencha apenas quando discordar da faixa proposta." type="list">
+    <dataValidation sqref="M2:M317" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use M0, M1, M2 ou Fora." promptTitle="Faixa revisada" prompt="Preencha apenas quando discordar da faixa proposta." type="list">
       <formula1>"M0,M1,M2,Fora"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N297" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Concorda com a faixa proposta?" prompt="Deixe em branco o que ainda não revisou." type="list">
+    <dataValidation sqref="N2:N317" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Concorda com a faixa proposta?" prompt="Deixe em branco o que ainda não revisou." type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16218,6 +17238,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F295" r:id="rId260"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F296" r:id="rId261"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F297" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F298" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F299" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F300" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F301" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F302" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F303" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F304" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F305" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F306" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F307" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F308" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F309" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F310" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F311" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F312" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F313" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F314" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F315" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F316" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F317" r:id="rId282"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16229,7 +17269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16956,26 +17996,58 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Operacional</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>PCONT</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Entrou no app em 29/10/2026 (AV-PC). Seis no M0, pelo critério: a empresa do grupo, a competência, a visão consolidada, o demonstrativo contra o ente, o ciclo recalcular–fechar–reabrir — que era da tela da Apuração e continua contado lá também — e as divergências com chamado, porque crédito que o ente não reconhece é crédito que falhou e precisa virar tratável. A guia do saldo, o ERP, o histórico e a auditoria ficam em M1: pagar o próprio saldo é obrigação a partir de 2027, mas a cadeia do crédito fecha sem a guia sair daqui — ela pode sair do portal. Três em M2, que explicam em vez de garantir: a simulação de parcial, os encargos e o painel executivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C24" s="15" t="n">
-        <v>116</v>
-      </c>
-      <c r="D24" s="15" t="n">
-        <v>143</v>
-      </c>
-      <c r="E24" s="15" t="n">
-        <v>35</v>
-      </c>
-      <c r="F24" s="15" t="n">
+      <c r="C25" s="15" t="n">
+        <v>122</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>154</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>38</v>
+      </c>
+      <c r="F25" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="15" t="n">
-        <v>296</v>
+      <c r="G25" s="15" t="n">
+        <v>316</v>
       </c>
     </row>
   </sheetData>
@@ -18261,7 +19333,7 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>v2.11</t>
+          <t>v2.12</t>
         </is>
       </c>
     </row>
@@ -18273,7 +19345,7 @@
       </c>
       <c r="B27" s="20" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
     </row>
@@ -18285,7 +19357,7 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Mapa de Funcionalidades v2.10</t>
+          <t>Mapa de Funcionalidades v2.11</t>
         </is>
       </c>
     </row>
@@ -18297,7 +19369,7 @@
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>296 funcionalidades · 21 módulos · 286 do mapa + 10 novas</t>
+          <t>316 funcionalidades · 22 módulos · 306 do mapa + 10 novas</t>
         </is>
       </c>
     </row>
@@ -18309,7 +19381,7 @@
       </c>
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>116 · 143 · 35 · 2</t>
+          <t>122 · 154 · 38 · 2</t>
         </is>
       </c>
     </row>

</xml_diff>